<commit_message>
Atualização do arquivo .gitignore para ignorar o arquivo temporário do projeto PCB e substituição dos arquivos PCB_Project.xlsx e Supply.SchDoc.
</commit_message>
<xml_diff>
--- a/Hardware/PCB_Project.xlsx
+++ b/Hardware/PCB_Project.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\NT-0967\Desktop\Arquivos\TCC\Hardware\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C629B71D-0AB9-4C8C-AEE8-3A6155C76FD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBF3DAA9-D8EE-4202-A8E8-2F277688FDE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20610" yWindow="-4800" windowWidth="20730" windowHeight="11160" xr2:uid="{D1BA460D-8128-452A-9C7C-0888C2394201}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{D1BA460D-8128-452A-9C7C-0888C2394201}"/>
   </bookViews>
   <sheets>
     <sheet name="PCB_Project" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="79">
   <si>
     <t>Designator</t>
   </si>
@@ -53,42 +53,18 @@
     <t>Quantity</t>
   </si>
   <si>
-    <t>C1</t>
-  </si>
-  <si>
-    <t>=Value</t>
-  </si>
-  <si>
-    <t>CAP ALUM 220UF 20% 63V RADIAL</t>
-  </si>
-  <si>
-    <t>C2, C3, C4, C5, C6</t>
-  </si>
-  <si>
     <t/>
   </si>
   <si>
     <t>C7, C8, C9</t>
   </si>
   <si>
-    <t>1 uF</t>
-  </si>
-  <si>
-    <t>Radial Leaded Multilayer Ceramic Capacitor, 0.1 uF, +/- 10%, 50 V, -55 to 125 degC, 2-Pin THD, RoHS, Tape and Reel</t>
-  </si>
-  <si>
     <t>C10, C12, C14</t>
   </si>
   <si>
-    <t>4.7 uF 50 V</t>
-  </si>
-  <si>
     <t>C11, C13, C15, C16, C17, C18, C19, C20, C21, C22, C23</t>
   </si>
   <si>
-    <t>0.1 uF 50 V</t>
-  </si>
-  <si>
     <t>D1, D4, D7</t>
   </si>
   <si>
@@ -128,21 +104,12 @@
     <t>Q1, Q2, Q3, Q4, Q5, Q6</t>
   </si>
   <si>
-    <t>=Part Number</t>
-  </si>
-  <si>
-    <t>MOSFET N CH 60V 240A D2PAK</t>
-  </si>
-  <si>
     <t>R1, R2, R3, R4, R5, R6, R7, R9, R12</t>
   </si>
   <si>
     <t>MFR-25FBF52-10R</t>
   </si>
   <si>
-    <t>Axial Resistor, 1 KOhm, +/- 1%, 250 mW, -55 to 155 degC, 2-Pin THD, RoHS, Bulk</t>
-  </si>
-  <si>
     <t>R8</t>
   </si>
   <si>
@@ -167,27 +134,9 @@
     <t>CSS2H-3920R-1L00F</t>
   </si>
   <si>
-    <t>RES 0.001 OHM 1% 8W 3920</t>
-  </si>
-  <si>
-    <t>U1</t>
-  </si>
-  <si>
-    <t>Buck Converver 15V</t>
-  </si>
-  <si>
-    <t>U2</t>
-  </si>
-  <si>
-    <t>Buck Converver 5V</t>
-  </si>
-  <si>
     <t>U3</t>
   </si>
   <si>
-    <t>DEVKIT_V1_ESP32-WROOM-32</t>
-  </si>
-  <si>
     <t>WROOM-32 Development Board ESP32 ESP-32S WiFi Bluetooth Dev Module</t>
   </si>
   <si>
@@ -197,38 +146,169 @@
     <t>IR2110PBF</t>
   </si>
   <si>
-    <t>High and Low Side Driver, All High Voltage Pins On One Side, Separate Logic and Power Ground, Shut-Down</t>
-  </si>
-  <si>
     <t>U7, U9, U10</t>
   </si>
   <si>
     <t>INA240A1DR</t>
   </si>
   <si>
-    <t>IC CURR SENSE 1 CIRCUIT 8SOIC</t>
-  </si>
-  <si>
     <t>U8</t>
   </si>
   <si>
     <t>LM339N</t>
   </si>
   <si>
-    <t>IC QUAD DIFF COMPARATOR 14-DIP</t>
+    <t>C1, C2, C3, C4, C5, C6</t>
+  </si>
+  <si>
+    <t>U1, U2</t>
+  </si>
+  <si>
+    <t>Step-Down Buck Converver LM2596</t>
+  </si>
+  <si>
+    <t>DEVKIT V1 ESP32-WROOM-32</t>
+  </si>
+  <si>
+    <t>UPW1J221MPD</t>
+  </si>
+  <si>
+    <t>1 µF ±10% 50V Ceramic Capacitor X7R Radial</t>
+  </si>
+  <si>
+    <t>C322C105K5R5TA</t>
+  </si>
+  <si>
+    <t>220 µF 63 V Aluminum Electrolytic Capacitors Radial, Can 5000 Hrs @ 105°C</t>
+  </si>
+  <si>
+    <t>C340C475K5R5TA</t>
+  </si>
+  <si>
+    <t>4.7 µF ±10% 50V Ceramic Capacitor X7R Radial</t>
+  </si>
+  <si>
+    <t>C320C104K5R5TA</t>
+  </si>
+  <si>
+    <t>0.1 µF ±10% 50V Ceramic Capacitor X7R Radial</t>
+  </si>
+  <si>
+    <t>IRFS7530-7PPBF</t>
+  </si>
+  <si>
+    <t>N-Channel 60 V 240A (Tc) 375W (Tc) Surface Mount D2PAK (7-Lead)</t>
+  </si>
+  <si>
+    <t>10 Ohms ±1% 0.25W, 1/4W Through Hole Resistor Axial Metal Film</t>
+  </si>
+  <si>
+    <t>39 kOhms ±1% 0.25W, 1/4W Through Hole Resistor Axial Metal Film</t>
+  </si>
+  <si>
+    <t>10 kOhms ±1% 0.25W, 1/4W Through Hole Resistor Axial Metal Film</t>
+  </si>
+  <si>
+    <t>4.7 kOhms ±1% 0.25W, 1/4W Through Hole Resistor Axial Metal Film</t>
+  </si>
+  <si>
+    <t>1 mOhms ±1% 8W Chip Resistor 3920 (1052 Metric) Automotive AEC-Q200, Current Sense Metal Element</t>
+  </si>
+  <si>
+    <t>Current Sense Amplifier 1 Circuit 8-SOIC</t>
+  </si>
+  <si>
+    <t>Comparator Standard (General Purpose) Open-Collector 14-PDIP</t>
+  </si>
+  <si>
+    <t>Half-Bridge Gate Driver IC Non-Inverting 14-DIP</t>
+  </si>
+  <si>
+    <t>110-93-314-41-001000</t>
+  </si>
+  <si>
+    <t>14 (2 x 7) Pos DIP, 0.3" (7.62mm) Row Spacing Socket Gold Through Hole</t>
+  </si>
+  <si>
+    <t>PPTC151LFBN-RC</t>
+  </si>
+  <si>
+    <t>15 Position Header Connector 0.100" (2.54mm) Through Hole Tin</t>
+  </si>
+  <si>
+    <t>Header</t>
+  </si>
+  <si>
+    <t>3132-10-1-0100-001-1-TS</t>
+  </si>
+  <si>
+    <t>10 AWG Hook-Up Wire 105/0.0100" Black 300V 100.0' (30.5m)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wire Black </t>
+  </si>
+  <si>
+    <t>Wire Red</t>
+  </si>
+  <si>
+    <t>3132-10-1-0100-004-1-TS</t>
+  </si>
+  <si>
+    <t>10 AWG Hook-Up Wire 105/0.0100" Red 300V 100.0' (30.5m)</t>
+  </si>
+  <si>
+    <t>Conectores Bullet Macho</t>
+  </si>
+  <si>
+    <t>Conectores Bullet Fêmea</t>
+  </si>
+  <si>
+    <t>Motor Brushless 4S</t>
+  </si>
+  <si>
+    <t>Controle de PS4</t>
+  </si>
+  <si>
+    <t>Placa de Fenolite 200mmX150mm</t>
+  </si>
+  <si>
+    <t>Carregador de bateria Lipo</t>
+  </si>
+  <si>
+    <t>Bateria LIPO 4S</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -272,12 +352,32 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -612,223 +712,224 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E7959FC3-FA30-4345-B94B-1C30DDBA7C2A}">
-  <dimension ref="A1:D22"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:D31"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="45" customWidth="1"/>
-    <col min="2" max="2" width="30" customWidth="1"/>
-    <col min="3" max="3" width="90" customWidth="1"/>
-    <col min="4" max="4" width="19" customWidth="1"/>
+    <col min="1" max="1" width="59.6640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="37.21875" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="108.21875" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="16384" width="8.88671875" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:4" s="1" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="8" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>4</v>
+        <v>39</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>5</v>
+        <v>43</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D2" s="3">
         <v>6</v>
-      </c>
-      <c r="D2" s="1">
-        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>8</v>
+        <v>45</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D3" s="1">
-        <v>5</v>
+        <v>44</v>
+      </c>
+      <c r="D3" s="3">
+        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>10</v>
+        <v>47</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D4" s="1">
+        <v>48</v>
+      </c>
+      <c r="D4" s="3">
         <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>13</v>
+        <v>49</v>
       </c>
       <c r="C5" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D5" s="3">
         <v>11</v>
-      </c>
-      <c r="D5" s="1">
-        <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D6" s="1">
-        <v>11</v>
+        <v>10</v>
+      </c>
+      <c r="D6" s="3">
+        <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D7" s="1">
-        <v>3</v>
+        <v>13</v>
+      </c>
+      <c r="D7" s="3">
+        <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D8" s="1">
-        <v>6</v>
+        <v>16</v>
+      </c>
+      <c r="D8" s="3">
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="D9" s="1">
+        <v>19</v>
+      </c>
+      <c r="D9" s="3">
         <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>26</v>
+        <v>51</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D10" s="1">
-        <v>1</v>
+        <v>52</v>
+      </c>
+      <c r="D10" s="3">
+        <v>6</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11" s="2" t="s">
-        <v>28</v>
+      <c r="A11" s="7" t="s">
+        <v>21</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="D11" s="1">
-        <v>6</v>
+        <v>53</v>
+      </c>
+      <c r="D11" s="3">
+        <v>9</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="D12" s="1">
-        <v>9</v>
+        <v>54</v>
+      </c>
+      <c r="D12" s="3">
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="D13" s="1">
-        <v>1</v>
+        <v>55</v>
+      </c>
+      <c r="D13" s="3">
+        <v>7</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="D14" s="1">
-        <v>7</v>
+        <v>56</v>
+      </c>
+      <c r="D14" s="3">
+        <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="D15" s="1">
-        <v>1</v>
+        <v>57</v>
+      </c>
+      <c r="D15" s="3">
+        <v>3</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
@@ -839,94 +940,159 @@
         <v>41</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="D16" s="1">
-        <v>3</v>
+        <v>4</v>
+      </c>
+      <c r="D16" s="3">
+        <v>2</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D17" s="1">
+        <v>32</v>
+      </c>
+      <c r="D17" s="3">
         <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D18" s="1">
-        <v>1</v>
+        <v>60</v>
+      </c>
+      <c r="D18" s="3">
+        <v>3</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
-        <v>47</v>
+        <v>35</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="D19" s="1">
-        <v>1</v>
+        <v>58</v>
+      </c>
+      <c r="D19" s="3">
+        <v>3</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
-        <v>50</v>
+        <v>37</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="D20" s="1">
-        <v>3</v>
+        <v>59</v>
+      </c>
+      <c r="D20" s="3">
+        <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A21" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="D21" s="1">
-        <v>3</v>
+      <c r="A21" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="D21" s="6">
+        <v>4</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A22" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="D22" s="1">
+      <c r="A22" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="D22" s="6">
         <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A23" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="D23" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A24" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="D24" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A25" s="4" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A26" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="B26" s="5"/>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A27" s="4" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A28" s="4" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A29" s="4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A30" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="B30" s="5"/>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A31" s="4" t="s">
+        <v>77</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização do arquivo PCB_Project.xlsx com novas alterações de projeto.
</commit_message>
<xml_diff>
--- a/Hardware/PCB_Project.xlsx
+++ b/Hardware/PCB_Project.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\NT-0967\Desktop\Arquivos\TCC\Hardware\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBF3DAA9-D8EE-4202-A8E8-2F277688FDE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90F654FD-D4B5-4548-AC74-C9834AC6CDA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{D1BA460D-8128-452A-9C7C-0888C2394201}"/>
+    <workbookView xWindow="-20610" yWindow="-4800" windowWidth="20730" windowHeight="11160" xr2:uid="{D1BA460D-8128-452A-9C7C-0888C2394201}"/>
   </bookViews>
   <sheets>
     <sheet name="PCB_Project" sheetId="1" r:id="rId1"/>
@@ -311,7 +311,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -324,8 +324,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -348,11 +354,107 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -366,23 +468,302 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="9">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFD3D3D3"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -393,6 +774,19 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{AC300413-4865-43EC-82D9-E313FD75FB18}" name="Tabela1" displayName="Tabela1" ref="A1:D31" totalsRowShown="0" headerRowDxfId="0" dataDxfId="8" headerRowBorderDxfId="6" tableBorderDxfId="7" totalsRowBorderDxfId="5">
+  <autoFilter ref="A1:D31" xr:uid="{AC300413-4865-43EC-82D9-E313FD75FB18}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{8D96E0ED-77C3-4226-9A44-F79F8E947519}" name="Designator" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{DF330E31-1B69-4A2A-8999-D50FDA3EF468}" name="Comment" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{3E59FC37-6986-492A-974D-C00D3990DEBF}" name="Description" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{0FDE8326-9725-4DB2-9CF9-76C6CEBE40D5}" name="Quantity" dataDxfId="1"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -715,10 +1109,10 @@
   <dimension ref="A1:D31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="59.6640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="37.21875" style="4" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="59.88671875" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="37.44140625" style="4" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="108.21875" style="4" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.6640625" style="4" bestFit="1" customWidth="1"/>
     <col min="5" max="16384" width="8.88671875" style="4"/>
   </cols>
   <sheetData>
@@ -726,18 +1120,18 @@
       <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="D1" s="9" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="10" t="s">
         <v>39</v>
       </c>
       <c r="B2" s="2" t="s">
@@ -746,12 +1140,12 @@
       <c r="C2" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="D2" s="3">
+      <c r="D2" s="11">
         <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="10" t="s">
         <v>5</v>
       </c>
       <c r="B3" s="2" t="s">
@@ -760,12 +1154,12 @@
       <c r="C3" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="D3" s="3">
+      <c r="D3" s="11">
         <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="10" t="s">
         <v>6</v>
       </c>
       <c r="B4" s="2" t="s">
@@ -774,12 +1168,12 @@
       <c r="C4" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="D4" s="3">
+      <c r="D4" s="11">
         <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="10" t="s">
         <v>7</v>
       </c>
       <c r="B5" s="2" t="s">
@@ -788,12 +1182,12 @@
       <c r="C5" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="D5" s="3">
+      <c r="D5" s="11">
         <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="10" t="s">
         <v>8</v>
       </c>
       <c r="B6" s="2" t="s">
@@ -802,12 +1196,12 @@
       <c r="C6" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="3">
+      <c r="D6" s="11">
         <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="10" t="s">
         <v>11</v>
       </c>
       <c r="B7" s="2" t="s">
@@ -816,12 +1210,12 @@
       <c r="C7" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D7" s="3">
+      <c r="D7" s="11">
         <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="10" t="s">
         <v>14</v>
       </c>
       <c r="B8" s="2" t="s">
@@ -830,12 +1224,12 @@
       <c r="C8" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="D8" s="3">
+      <c r="D8" s="11">
         <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="10" t="s">
         <v>17</v>
       </c>
       <c r="B9" s="2" t="s">
@@ -844,26 +1238,26 @@
       <c r="C9" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D9" s="3">
+      <c r="D9" s="11">
         <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="D10" s="3">
+      <c r="D10" s="13">
         <v>6</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11" s="7" t="s">
+      <c r="A11" s="14" t="s">
         <v>21</v>
       </c>
       <c r="B11" s="2" t="s">
@@ -872,12 +1266,12 @@
       <c r="C11" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="D11" s="3">
+      <c r="D11" s="11">
         <v>9</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="10" t="s">
         <v>23</v>
       </c>
       <c r="B12" s="2" t="s">
@@ -886,12 +1280,12 @@
       <c r="C12" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="D12" s="3">
+      <c r="D12" s="11">
         <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13" s="2" t="s">
+      <c r="A13" s="10" t="s">
         <v>25</v>
       </c>
       <c r="B13" s="2" t="s">
@@ -900,12 +1294,12 @@
       <c r="C13" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="D13" s="3">
+      <c r="D13" s="11">
         <v>7</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A14" s="2" t="s">
+      <c r="A14" s="10" t="s">
         <v>27</v>
       </c>
       <c r="B14" s="2" t="s">
@@ -914,12 +1308,12 @@
       <c r="C14" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="D14" s="3">
+      <c r="D14" s="11">
         <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A15" s="2" t="s">
+      <c r="A15" s="10" t="s">
         <v>29</v>
       </c>
       <c r="B15" s="2" t="s">
@@ -928,54 +1322,54 @@
       <c r="C15" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="D15" s="3">
+      <c r="D15" s="11">
         <v>3</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A16" s="2" t="s">
+      <c r="A16" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="C16" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D16" s="3">
+      <c r="D16" s="13">
         <v>2</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A17" s="2" t="s">
+      <c r="A17" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B17" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="C17" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="D17" s="3">
+      <c r="D17" s="13">
         <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A18" s="2" t="s">
+      <c r="A18" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B18" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="C18" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="D18" s="3">
+      <c r="D18" s="13">
         <v>3</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A19" s="2" t="s">
+      <c r="A19" s="10" t="s">
         <v>35</v>
       </c>
       <c r="B19" s="2" t="s">
@@ -984,12 +1378,12 @@
       <c r="C19" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="D19" s="3">
+      <c r="D19" s="11">
         <v>3</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A20" s="2" t="s">
+      <c r="A20" s="10" t="s">
         <v>37</v>
       </c>
       <c r="B20" s="2" t="s">
@@ -998,12 +1392,12 @@
       <c r="C20" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D20" s="3">
+      <c r="D20" s="11">
         <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A21" s="6" t="s">
+      <c r="A21" s="15" t="s">
         <v>65</v>
       </c>
       <c r="B21" s="3" t="s">
@@ -1012,12 +1406,12 @@
       <c r="C21" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="D21" s="6">
+      <c r="D21" s="11">
         <v>4</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A22" s="6" t="s">
+      <c r="A22" s="15" t="s">
         <v>65</v>
       </c>
       <c r="B22" s="3" t="s">
@@ -1026,12 +1420,12 @@
       <c r="C22" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="D22" s="6">
+      <c r="D22" s="11">
         <v>1</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A23" s="6" t="s">
+      <c r="A23" s="15" t="s">
         <v>68</v>
       </c>
       <c r="B23" s="3" t="s">
@@ -1040,12 +1434,12 @@
       <c r="C23" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="D23" s="6">
+      <c r="D23" s="11">
         <v>1</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A24" s="3" t="s">
+      <c r="A24" s="15" t="s">
         <v>69</v>
       </c>
       <c r="B24" s="3" t="s">
@@ -1054,49 +1448,85 @@
       <c r="C24" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="D24" s="6">
+      <c r="D24" s="11">
         <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A25" s="4" t="s">
+      <c r="A25" s="15" t="s">
         <v>72</v>
       </c>
+      <c r="B25" s="3"/>
+      <c r="C25" s="3"/>
+      <c r="D25" s="11">
+        <v>3</v>
+      </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A26" s="4" t="s">
+      <c r="A26" s="15" t="s">
         <v>73</v>
       </c>
-      <c r="B26" s="5"/>
+      <c r="B26" s="16"/>
+      <c r="C26" s="3"/>
+      <c r="D26" s="11">
+        <v>3</v>
+      </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A27" s="4" t="s">
+      <c r="A27" s="15" t="s">
         <v>78</v>
       </c>
+      <c r="B27" s="3"/>
+      <c r="C27" s="3"/>
+      <c r="D27" s="11">
+        <v>1</v>
+      </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A28" s="4" t="s">
+      <c r="A28" s="15" t="s">
         <v>74</v>
       </c>
+      <c r="B28" s="3"/>
+      <c r="C28" s="3"/>
+      <c r="D28" s="11">
+        <v>1</v>
+      </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A29" s="4" t="s">
+      <c r="A29" s="20" t="s">
         <v>75</v>
       </c>
+      <c r="B29" s="6"/>
+      <c r="C29" s="6"/>
+      <c r="D29" s="13">
+        <v>1</v>
+      </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A30" s="4" t="s">
+      <c r="A30" s="15" t="s">
         <v>76</v>
       </c>
-      <c r="B30" s="5"/>
+      <c r="B30" s="16"/>
+      <c r="C30" s="3"/>
+      <c r="D30" s="11">
+        <v>1</v>
+      </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A31" s="4" t="s">
+      <c r="A31" s="17" t="s">
         <v>77</v>
+      </c>
+      <c r="B31" s="18"/>
+      <c r="C31" s="18"/>
+      <c r="D31" s="19">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>